<commit_message>
Load maker photos from the images folder
Photo columns in the sheet can now hold a plain file name that loads
from images/ in this repo. Full links and Google Drive links still work.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YSqo5Gce3Bof2cSdRCMead
</commit_message>
<xml_diff>
--- a/sheet-template.xlsx
+++ b/sheet-template.xlsx
@@ -516,7 +516,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>• photo_1 to photo_3: paste a Google Drive share link (file must be shared 'Anyone with the link') or any direct image link. At least one per maker.</t>
+          <t>• photo_1 to photo_3: upload the photo to the images folder in the GitHub repo, then type its file name here exactly, e.g. harbour-prints-1.jpg. At least one per maker. (A full https:// image link also works.)</t>
         </is>
       </c>
     </row>
@@ -744,7 +744,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/PASTE-FILE-ID/view</t>
+          <t>example-ceramics-1.jpg</t>
         </is>
       </c>
       <c r="F2" s="5" t="inlineStr"/>

</xml_diff>